<commit_message>
updated read and write logic for excel
</commit_message>
<xml_diff>
--- a/datasheet.xlsx
+++ b/datasheet.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42872E7E-8194-4BE9-8472-8387A2CFB560}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC06F719-CE51-4023-B540-308AC5370686}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="login" sheetId="1" r:id="rId1"/>
-    <sheet name="usercreation" sheetId="2" r:id="rId2"/>
+    <sheet name="userCreation" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="67">
   <si>
     <t>Admin</t>
   </si>
@@ -45,18 +45,18 @@
     <t>admin1234</t>
   </si>
   <si>
+    <t>First Name</t>
+  </si>
+  <si>
+    <t>Middle Name</t>
+  </si>
+  <si>
+    <t>LastName</t>
+  </si>
+  <si>
     <t>EmployeeId</t>
   </si>
   <si>
-    <t>First Name</t>
-  </si>
-  <si>
-    <t>Middle Name</t>
-  </si>
-  <si>
-    <t>LastName</t>
-  </si>
-  <si>
     <t xml:space="preserve">Toggle On </t>
   </si>
   <si>
@@ -70,14 +70,169 @@
   </si>
   <si>
     <t>Upload image</t>
+  </si>
+  <si>
+    <t>John</t>
+  </si>
+  <si>
+    <t>Doe</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>John.doe123</t>
+  </si>
+  <si>
+    <t>Enabled</t>
+  </si>
+  <si>
+    <t>Manju@1234</t>
+  </si>
+  <si>
+    <t>testdata/test1.jpg</t>
+  </si>
+  <si>
+    <t>S.No</t>
+  </si>
+  <si>
+    <t>ScenarioType</t>
+  </si>
+  <si>
+    <t>ExecuteFlag</t>
+  </si>
+  <si>
+    <t>Test case status</t>
+  </si>
+  <si>
+    <t>Successfully Saved</t>
+  </si>
+  <si>
+    <t>Positive</t>
+  </si>
+  <si>
+    <t>Steve</t>
+  </si>
+  <si>
+    <t>Peter</t>
+  </si>
+  <si>
+    <t>James</t>
+  </si>
+  <si>
+    <t>Parker</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Negative</t>
+  </si>
+  <si>
+    <t>Required</t>
+  </si>
+  <si>
+    <t>David</t>
+  </si>
+  <si>
+    <t>Smith</t>
+  </si>
+  <si>
+    <t>Lee</t>
+  </si>
+  <si>
+    <t>Already Exists</t>
+  </si>
+  <si>
+    <t>Harry</t>
+  </si>
+  <si>
+    <t>Potter</t>
+  </si>
+  <si>
+    <t>Harry123</t>
+  </si>
+  <si>
+    <t>Test@1234</t>
+  </si>
+  <si>
+    <t>Passwords Do Not Match</t>
+  </si>
+  <si>
+    <t>Robert</t>
+  </si>
+  <si>
+    <t>Downey</t>
+  </si>
+  <si>
+    <t>Robert123</t>
+  </si>
+  <si>
+    <t>Password Must Meet Complexity Requirements</t>
+  </si>
+  <si>
+    <t>Clark</t>
+  </si>
+  <si>
+    <t>Kent</t>
+  </si>
+  <si>
+    <t>Superman</t>
+  </si>
+  <si>
+    <t>EMP1001</t>
+  </si>
+  <si>
+    <t>Clark001</t>
+  </si>
+  <si>
+    <t>Disabled</t>
+  </si>
+  <si>
+    <t>Bruce</t>
+  </si>
+  <si>
+    <t>Wayne</t>
+  </si>
+  <si>
+    <t>Batman</t>
+  </si>
+  <si>
+    <t>Employee Id Already Exists</t>
+  </si>
+  <si>
+    <t>Tony</t>
+  </si>
+  <si>
+    <t>Stark</t>
+  </si>
+  <si>
+    <t>Ironman</t>
+  </si>
+  <si>
+    <t>Tony@123</t>
+  </si>
+  <si>
+    <t>testdata/test.pdf</t>
+  </si>
+  <si>
+    <t>Invalid File Type</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -111,9 +266,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -464,50 +623,467 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16313A00-36E6-4ECF-BA1E-C9D31747B485}">
-  <dimension ref="A1:K1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:P11"/>
+  <sheetFormatPr defaultRowHeight="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.88671875" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="5" max="5" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.5546875" customWidth="1"/>
+    <col min="8" max="8" width="15.33203125" customWidth="1"/>
+    <col min="9" max="9" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="7.88671875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="40.109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="14.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B1" t="s">
+      <c r="F1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C1" t="s">
+      <c r="G1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D1" t="s">
+      <c r="H1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+      <c r="K3" s="2"/>
+      <c r="L3" s="2"/>
+      <c r="M3" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+      <c r="K4" s="2"/>
+      <c r="L4" s="2"/>
+      <c r="M4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N4" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="2">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="I5" s="2"/>
+      <c r="J5" s="2"/>
+      <c r="K5" s="2"/>
+      <c r="L5" s="2"/>
+      <c r="M5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N5" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="2">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="M6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N6" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="2">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="M7" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N7" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="2">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K8" s="2">
+        <v>123</v>
+      </c>
+      <c r="L8" s="2">
+        <v>123</v>
+      </c>
+      <c r="M8" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N8" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="2">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="L9" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="M9" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N9" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="2">
         <v>9</v>
       </c>
-      <c r="E1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F1" t="s">
-        <v>14</v>
-      </c>
-      <c r="G1" t="s">
-        <v>15</v>
-      </c>
-      <c r="H1" t="s">
-        <v>1</v>
-      </c>
-      <c r="I1" t="s">
-        <v>16</v>
-      </c>
-      <c r="K1" t="s">
-        <v>17</v>
+      <c r="B10" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="I10" s="2"/>
+      <c r="J10" s="2"/>
+      <c r="K10" s="2"/>
+      <c r="L10" s="2"/>
+      <c r="M10" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N10" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="2">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="M11" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="N11" s="2" t="s">
+        <v>66</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>